<commit_message>
feat(pt-BR): fecha as 62 dúvidas do PO (PENDENTE_PO 62 -> 0)
CORRECOES_PO: 62 decisões vinculativas (grupos A glossário, B sem tradução
na fonte, C vazios). Uma decisão de PO tem precedência sobre o aviso da
fonte e sobre as decisões dos agentes, fechando a linha como CORRIGIDO.

- FALSE_POSITIVOS_PT_PT isenta 'Fatura anulada' (INVCVOID) da porta
  automática de resíduo: mantém a distinção BR fiscal anulada != cancelada.
- regras 'fatura anulada(s)->fatura cancelada(s)' removidas (contradiziam a
  decisão fiscal); o converter continua a tratar 'anulado/anular' em geral.
- DUVIDAS_KEYS/DUVIDAS_GRUPOS esvaziados; duvidas_PO.xlsx sem linhas.
- testes: 74 OK; QA sign-off PASS (amostra 5%: 0/285 reprovadas).
- contagem: OK 15231 | CORRIGIDO 4408 | PENDENTE_PO 0 | total 19639.
</commit_message>
<xml_diff>
--- a/duvidas_PO.xlsx
+++ b/duvidas_PO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,230 +445,6 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>Destino</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>apps.aiAssistant.label.hotel</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hotel</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>D4 aiAssistant hotel/property</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>apps.chainSpaceLockType.radio.onHold</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>OnHold (Ative esta opção para bloquear o alojamento)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>D3 OnHold/OutOfOrder/OutOfService</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>apps.chainSpaceLockType.radio.outOfOrder</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>OutOfOrder (Ative esta opção para permitir retirar o alojamento do inventário)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>D3 OnHold/OutOfOrder/OutOfService</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>apps.chainSpaceLockType.radio.outOfService</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>OutOfService (Ative esta opção para permitir retirar o alojamento da disponibilidade)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>D3 OnHold/OutOfOrder/OutOfService</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>core.label.billing</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Faturação</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>glossário</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>core.label.chain</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Cadeia</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>glossário</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>shared.forecast.nonDeductedAllotment</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Frontend (pantallas)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Allotment não deduzido</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>D2 allotment</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PropertyClassType t WHERE t.Code = '9'</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Entidades de sistema</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Pensão</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>D1 pensão/regime</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PO</t>
         </is>
       </c>
     </row>

</xml_diff>